<commit_message>
Update requirements and fix build error
</commit_message>
<xml_diff>
--- a/history.xlsx
+++ b/history.xlsx
@@ -809,6 +809,63 @@
 </file>
 
 <file path=xl/charts/chart20.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Distribution of Checked Messages</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <pieChart>
+        <varyColors val="1"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'History'!F1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'History'!$E$2:$E$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'History'!$F$2:$F$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <firstSliceAng val="0"/>
+      </pieChart>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart21.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -1706,6 +1763,28 @@
     </graphicFrame>
     <clientData/>
   </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="2700000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="21" name="Chart 21"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId21"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
 </wsDr>
 </file>
 
@@ -1998,7 +2077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2060,7 +2139,7 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4">
@@ -2393,6 +2472,23 @@
       <c r="C23" t="inlineStr">
         <is>
           <t>2026-01-11 09:47:52</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Don't forget to bring your notebook</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Not Spam ✅</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>2026-03-29 16:51:29</t>
         </is>
       </c>
     </row>

</xml_diff>